<commit_message>
Add arm disarm button support
</commit_message>
<xml_diff>
--- a/Requirements/Requirement.xlsx
+++ b/Requirements/Requirement.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Embedded_work\PROJECTS\PIR_Security_Node\Requirements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20FB2169-8EF4-4171-8F06-9DDE432DF704}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E06E596C-388A-4858-845E-8E8CC5F3392D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="16">
   <si>
     <t>ID</t>
   </si>
@@ -70,6 +70,9 @@
   </si>
   <si>
     <t>Not Started</t>
+  </si>
+  <si>
+    <t>Done</t>
   </si>
 </sst>
 </file>
@@ -403,7 +406,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.109375" customWidth="1"/>
-    <col min="2" max="2" width="13.88671875" customWidth="1"/>
+    <col min="2" max="2" width="25.6640625" customWidth="1"/>
     <col min="3" max="3" width="17.77734375" customWidth="1"/>
     <col min="4" max="4" width="18.6640625" customWidth="1"/>
   </cols>
@@ -433,7 +436,7 @@
         <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>